<commit_message>
fix: make scope-check workbook open directly in Excel
Remove sheet/workbook protection, comments, and invalid single-cell
merges that blocked editing or triggered Excel repair on open.

Co-authored-by: iremalisan <iremalisan@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Su_Verimliligi_Kapsam_Kontrol.xlsx
+++ b/Su_Verimliligi_Kapsam_Kontrol.xlsx
@@ -2,7 +2,6 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
@@ -263,17 +262,14 @@
     <xf numFmtId="0" fontId="1" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -451,21 +447,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Kapsam Tablosu</author>
-  </authors>
-  <commentList>
-    <comment ref="I9" authorId="0" shapeId="0">
-      <text>
-        <t>Bu sütun girilen NACE kodunu 4 haneye çevirir (10.11.01 → 10.11). Silmeyin.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2424,7 +2405,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="0" password="CE4B"/>
   <autoFilter ref="A9:I59"/>
   <mergeCells count="11">
     <mergeCell ref="A5:I5"/>
@@ -2473,7 +2453,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -6222,7 +6201,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <autoFilter ref="A1:E149"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -6338,10 +6316,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>